<commit_message>
Corrected reporting of energy commodity related flow cost so that they now both includes val_flo (market value of commodity) and cst_floc (commodity and proces specific delivery costs)
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_Z_TIMESReport.xlsx
+++ b/SuppXLS/Scen_Z_TIMESReport.xlsx
@@ -392,7 +392,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249880000948906"/>
+        <fgColor theme="0" tint="-0.249870002269745"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -410,7 +410,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249970003962517"/>
+        <fgColor theme="0" tint="-0.249960005283356"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>

</xml_diff>